<commit_message>
fix url typo (#1350)
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.jones\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6254447E-05CB-4F42-9A59-2EF72F312BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861FC0BE-4D7D-4629-A85C-7EE4E4DECCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -562,11 +562,15 @@
       <c r="B2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="C2" s="7">
+        <v>298</v>
+      </c>
+      <c r="D2" s="7">
+        <v>108</v>
+      </c>
       <c r="E2" s="8">
         <f t="shared" ref="E2:E28" si="0">IF(C2=0,0,+(C2-D2)/C2)</f>
-        <v>0</v>
+        <v>0.63758389261744963</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -691,9 +695,7 @@
       <c r="A10" s="5">
         <v>46123</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>14</v>
-      </c>
+      <c r="B10" s="13"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="8">
@@ -903,9 +905,8 @@
     <hyperlink ref="B7" r:id="rId6" display="https://sqlsaturday.com/2026-04-18-sqlsaturday1140/" xr:uid="{58E6D6B4-5ED4-4714-8FDB-E08CF0662BC3}"/>
     <hyperlink ref="B8" r:id="rId7" display="https://sqlsaturday.com/2026-03-28-sqlsaturday1142/" xr:uid="{437241E0-0AAF-4D4E-8A16-325412A2DA23}"/>
     <hyperlink ref="B9" r:id="rId8" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1135/" xr:uid="{0D895616-7215-4314-966E-B2E806332540}"/>
-    <hyperlink ref="B10" r:id="rId9" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1139/" xr:uid="{6A71CCDA-7470-4C2B-A96E-07211211B3F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
austin new event  #1361
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.jones\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539A48E6-B8B9-4BB3-817B-E1DB5CF6B3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2CEFEF-6379-46B5-855A-14149B8CABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="300" windowWidth="24465" windowHeight="15315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Date</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t>Houston Ai-Lytics Day 2026 (#1137)</t>
+  </si>
+  <si>
+    <t>SQL Saturday Arequipa 2026 (#1147)</t>
+  </si>
+  <si>
+    <t>Day of Data Jacksonville 2026 (#1128) </t>
+  </si>
+  <si>
+    <t>SQL Saturday Haiti 2026 (#1145) - Virtual -</t>
   </si>
 </sst>
 </file>
@@ -519,17 +528,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,7 +567,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>46039</v>
       </c>
@@ -576,7 +585,7 @@
         <v>0.63758389261744963</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>46256</v>
       </c>
@@ -590,7 +599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>46102</v>
       </c>
@@ -608,7 +617,7 @@
         <v>0.44612068965517243</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>46123</v>
       </c>
@@ -626,7 +635,7 @@
         <v>0.42514970059880242</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>46123</v>
       </c>
@@ -644,7 +653,7 @@
         <v>0.33823529411764708</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="16">
         <v>46130</v>
       </c>
@@ -658,7 +667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>46109</v>
       </c>
@@ -676,7 +685,7 @@
         <v>9.0909090909090912E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>46123</v>
       </c>
@@ -694,19 +703,25 @@
         <v>0.42514970059880242</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46123</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+        <v>46137</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="7">
+        <v>46</v>
+      </c>
+      <c r="D10" s="7">
+        <v>42</v>
+      </c>
       <c r="E10" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.6956521739130432E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>46137</v>
       </c>
@@ -724,9 +739,13 @@
         <v>7.0512820512820512E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6"/>
+    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>46144</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>20</v>
+      </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="8">
@@ -734,9 +753,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6"/>
+    <row r="13" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8">
@@ -744,7 +767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
@@ -754,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
@@ -764,7 +787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="E16" s="8">
@@ -772,7 +795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="E17" s="8">
@@ -780,7 +803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="E18" s="8">
@@ -791,7 +814,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19" s="8">
@@ -799,7 +822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20"/>
       <c r="D20"/>
       <c r="E20" s="8">
@@ -807,7 +830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21" s="8">
@@ -815,7 +838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="13"/>
       <c r="E22" s="8">
@@ -823,7 +846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="13"/>
       <c r="E23" s="8">
@@ -831,7 +854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="13"/>
       <c r="E24" s="8">
@@ -839,7 +862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="13"/>
       <c r="E25" s="8">
@@ -847,7 +870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="13"/>
       <c r="E26" s="8">
@@ -855,7 +878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="13"/>
       <c r="E27" s="8">
@@ -863,7 +886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="13"/>
       <c r="E28" s="8">
@@ -871,37 +894,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="13"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="14"/>
       <c r="E30" s="8"/>
     </row>
-    <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="10"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="10"/>
       <c r="E32" s="8"/>
     </row>
-    <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="10"/>
       <c r="E33" s="8"/>
     </row>
-    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="10"/>
       <c r="E34" s="8"/>
     </row>
-    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="10"/>
       <c r="E35" s="8"/>
@@ -917,8 +940,11 @@
     <hyperlink ref="B8" r:id="rId7" display="https://sqlsaturday.com/2026-03-28-sqlsaturday1142/" xr:uid="{437241E0-0AAF-4D4E-8A16-325412A2DA23}"/>
     <hyperlink ref="B9" r:id="rId8" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1135/" xr:uid="{0D895616-7215-4314-966E-B2E806332540}"/>
     <hyperlink ref="B11" r:id="rId9" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1137/" xr:uid="{CBF1FDBB-4936-434E-A18B-A7006D90C96F}"/>
+    <hyperlink ref="B10" r:id="rId10" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1147/" xr:uid="{52A6CAD9-6FF4-4021-AF96-9A11F100CAB7}"/>
+    <hyperlink ref="B12" r:id="rId11" display="https://sqlsaturday.com/2026-05-02-sqlsaturday1128/" xr:uid="{C267197A-EBDF-43AC-A57A-47836385B40A}"/>
+    <hyperlink ref="B13" r:id="rId12" display="https://sqlsaturday.com/2026-05-16-sqlsaturday1145/" xr:uid="{7DE4CF3A-72E8-4101-9C80-B98C8F772699}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
austin new event  #1361 (#1362)
* austin new event  #1361

* added attendance updates
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.jones\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539A48E6-B8B9-4BB3-817B-E1DB5CF6B3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47FD44D8-8219-41AA-8473-DA96CFE00685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="300" windowWidth="24465" windowHeight="15315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Attendance" sheetId="1" r:id="rId1"/>
+    <sheet name="Jobs" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -90,6 +91,33 @@
   </si>
   <si>
     <t>Houston Ai-Lytics Day 2026 (#1137)</t>
+  </si>
+  <si>
+    <t>SQL Saturday Arequipa 2026 (#1147)</t>
+  </si>
+  <si>
+    <t>Day of Data Jacksonville 2026 (#1128) </t>
+  </si>
+  <si>
+    <t>SQL Saturday Haiti 2026 (#1145) - Virtual -</t>
+  </si>
+  <si>
+    <t>App Developers</t>
+  </si>
+  <si>
+    <t>Architects</t>
+  </si>
+  <si>
+    <t>DBA</t>
+  </si>
+  <si>
+    <t>Data Engineer</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -170,7 +198,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -211,6 +239,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -519,17 +550,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,7 +589,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>46039</v>
       </c>
@@ -576,7 +607,7 @@
         <v>0.63758389261744963</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>46256</v>
       </c>
@@ -590,7 +621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>46102</v>
       </c>
@@ -608,7 +639,7 @@
         <v>0.44612068965517243</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>46123</v>
       </c>
@@ -626,7 +657,7 @@
         <v>0.42514970059880242</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>46123</v>
       </c>
@@ -644,7 +675,7 @@
         <v>0.33823529411764708</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="16">
         <v>46130</v>
       </c>
@@ -658,7 +689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>46109</v>
       </c>
@@ -676,7 +707,7 @@
         <v>9.0909090909090912E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>46123</v>
       </c>
@@ -694,19 +725,25 @@
         <v>0.42514970059880242</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46123</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+        <v>46137</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="7">
+        <v>46</v>
+      </c>
+      <c r="D10" s="7">
+        <v>42</v>
+      </c>
       <c r="E10" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.6956521739130432E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>46137</v>
       </c>
@@ -724,19 +761,31 @@
         <v>7.0512820512820512E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
+    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>46144</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="7">
+        <v>534</v>
+      </c>
+      <c r="D12" s="7">
+        <v>371</v>
+      </c>
       <c r="E12" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6"/>
+        <v>0.30524344569288392</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8">
@@ -744,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
@@ -754,7 +803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
@@ -764,7 +813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="E16" s="8">
@@ -772,7 +821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="E17" s="8">
@@ -780,7 +829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="E18" s="8">
@@ -791,7 +840,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19" s="8">
@@ -799,7 +848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20"/>
       <c r="D20"/>
       <c r="E20" s="8">
@@ -807,7 +856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21" s="8">
@@ -815,7 +864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="13"/>
       <c r="E22" s="8">
@@ -823,7 +872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="13"/>
       <c r="E23" s="8">
@@ -831,7 +880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="13"/>
       <c r="E24" s="8">
@@ -839,7 +888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="13"/>
       <c r="E25" s="8">
@@ -847,7 +896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="13"/>
       <c r="E26" s="8">
@@ -855,7 +904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="13"/>
       <c r="E27" s="8">
@@ -863,7 +912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="13"/>
       <c r="E28" s="8">
@@ -871,37 +920,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="13"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="14"/>
       <c r="E30" s="8"/>
     </row>
-    <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="10"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="10"/>
       <c r="E32" s="8"/>
     </row>
-    <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="10"/>
       <c r="E33" s="8"/>
     </row>
-    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="10"/>
       <c r="E34" s="8"/>
     </row>
-    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="10"/>
       <c r="E35" s="8"/>
@@ -917,8 +966,186 @@
     <hyperlink ref="B8" r:id="rId7" display="https://sqlsaturday.com/2026-03-28-sqlsaturday1142/" xr:uid="{437241E0-0AAF-4D4E-8A16-325412A2DA23}"/>
     <hyperlink ref="B9" r:id="rId8" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1135/" xr:uid="{0D895616-7215-4314-966E-B2E806332540}"/>
     <hyperlink ref="B11" r:id="rId9" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1137/" xr:uid="{CBF1FDBB-4936-434E-A18B-A7006D90C96F}"/>
+    <hyperlink ref="B10" r:id="rId10" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1147/" xr:uid="{52A6CAD9-6FF4-4021-AF96-9A11F100CAB7}"/>
+    <hyperlink ref="B12" r:id="rId11" display="https://sqlsaturday.com/2026-05-02-sqlsaturday1128/" xr:uid="{C267197A-EBDF-43AC-A57A-47836385B40A}"/>
+    <hyperlink ref="B13" r:id="rId12" display="https://sqlsaturday.com/2026-05-16-sqlsaturday1145/" xr:uid="{7DE4CF3A-72E8-4101-9C80-B98C8F772699}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808A6323-B2BF-43D1-9683-02EA2191A089}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="16.36328125" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" customWidth="1"/>
+    <col min="6" max="6" width="15.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>46039</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="5">
+        <v>46256</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
+        <v>46102</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="17">
+        <v>46130</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>46109</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>46137</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10">
+        <v>24</v>
+      </c>
+      <c r="G10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>46137</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>46144</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>53</v>
+      </c>
+      <c r="D12">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>45</v>
+      </c>
+      <c r="F12">
+        <v>106</v>
+      </c>
+      <c r="G12">
+        <v>25</v>
+      </c>
+      <c r="H12">
+        <f>26+25+27+35+36+53</f>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://sqlsaturday.com/2026-01-17-sqlsaturday1138/" xr:uid="{9BBFD336-5B49-4106-BC82-48F7FFABB181}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://sqlsaturday.com/2026-02-28-sqlsaturday1132/" xr:uid="{14C4551B-AA3E-4854-A92B-107A1E3BF749}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://sqlsaturday.com/2026-03-21-sqlsaturday1127/" xr:uid="{F69FEBB5-069E-4C66-B75B-65A012C62472}"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1135/" xr:uid="{8B84D329-68E7-4FFB-8C69-5324DD0D507F}"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1139/" xr:uid="{702A258F-A47A-449A-93A2-03B9D0A0FE5B}"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://sqlsaturday.com/2026-04-18-sqlsaturday1140/" xr:uid="{13A062FC-4BB7-410F-BC60-3CCF509AEAD9}"/>
+    <hyperlink ref="B8" r:id="rId7" display="https://sqlsaturday.com/2026-03-28-sqlsaturday1142/" xr:uid="{DF840437-E1D6-4D9E-A7F8-BE10A89F7E2F}"/>
+    <hyperlink ref="B9" r:id="rId8" display="https://sqlsaturday.com/2026-04-11-sqlsaturday1135/" xr:uid="{2CE9A7B7-C3DC-4953-915F-CBEE0F466C68}"/>
+    <hyperlink ref="B11" r:id="rId9" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1137/" xr:uid="{0878FD0D-0661-4DB7-AF7D-D259D14FB142}"/>
+    <hyperlink ref="B10" r:id="rId10" display="https://sqlsaturday.com/2026-04-25-sqlsaturday1147/" xr:uid="{2C514026-1108-4AEB-8461-B9A1F2D310C3}"/>
+    <hyperlink ref="B12" r:id="rId11" display="https://sqlsaturday.com/2026-05-02-sqlsaturday1128/" xr:uid="{97D3C2E9-D00E-4F8C-BD01-85CF5D6C0A48}"/>
+    <hyperlink ref="B13" r:id="rId12" display="https://sqlsaturday.com/2026-05-16-sqlsaturday1145/" xr:uid="{F6225BAC-FC20-4114-BB21-C62C7006DBDF}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated raleigh attendace (#1402)
Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance.xlsx
+++ b/assets/misc/2026/2026_Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAD9E81-0EDB-42A6-BA34-AB1FF6BA8371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFBF676-1384-4E42-9A5C-A73B70B8A893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24150" yWindow="225" windowWidth="24180" windowHeight="14175" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25845" yWindow="630" windowWidth="22860" windowHeight="13890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -833,14 +833,14 @@
         <v>27</v>
       </c>
       <c r="C13" s="6">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="D13" s="6">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5393258426966292</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1530,11 +1530,11 @@
       </c>
       <c r="G13" s="8">
         <f t="shared" ref="G13:G24" si="3">+H13-SUM(C13:F13)</f>
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="H13" s="8">
         <f>+Attendance!C13</f>
-        <v>0</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>